<commit_message>
docs(spec): SUP-002 升 V1.1——综合 Sprint 1.9 现状/三源种子/绑定裁决，新增 §0 实施对齐与 PC-OPEN-06/07
PPG 种子 V2：NPS 26/28/30/32/34→DN650-850 映射补齐（U4 DN700-850、P2 DN650-900
大口径段 V1 丢失修复，含 EFW 分段 SCH10 注记）；附录 A 按源文档修正
（U4 大口径 STD 非 10、分段材料）；开发计划 P2§2.5/P3§3.4 增补实施依据与阻塞关系。
</commit_message>
<xml_diff>
--- a/pcs-backend/app/seeds/pipe_classes_ppg.xlsx
+++ b/pcs-backend/app/seeds/pipe_classes_ppg.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "XS", "80": "STD", "100": "STD", "150": "STD", "200": "STD"}</t>
+          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "XS", "80": "STD", "100": "STD", "125": "STD", "150": "STD", "200": "STD"}</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "150": "STD"}</t>
+          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "125": "STD", "150": "STD"}</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "150": "STD", "200": "STD", "250": "STD", "300": "STD"}</t>
+          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "125": "STD", "150": "STD", "200": "STD", "250": "STD", "300": "STD"}</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "150": "STD", "200": "STD", "250": "STD", "300": "STD", "350": "STD", "400": "STD", "450": "STD", "500": "STD", "600": "STD", "900": "STD"}</t>
+          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "125": "STD", "150": "STD", "200": "STD", "250": "STD", "300": "STD", "350": "STD", "400": "STD", "450": "STD", "500": "STD", "600": "STD", "650": "STD", "700": "STD", "750": "STD", "800": "STD", "850": "STD", "900": "STD"}</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "150": "STD", "200": "STD", "250": "STD", "300": "Sch40"}</t>
+          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "125": "STD", "150": "STD", "200": "STD", "250": "STD", "300": "Sch40"}</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "150": "STD", "200": "STD", "250": "STD", "300": "STD"}</t>
+          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "125": "STD", "150": "STD", "200": "STD", "250": "STD", "300": "STD"}</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "XS", "80": "STD", "100": "STD", "150": "STD", "200": "STD"}</t>
+          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "XS", "80": "STD", "100": "STD", "125": "STD", "150": "STD", "200": "STD"}</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "150": "STD", "200": "STD", "250": "STD", "300": "STD"}</t>
+          <t>{"15": "XS", "20": "XS", "25": "XS", "32": "XS", "40": "XS", "50": "STD", "65": "STD", "80": "STD", "100": "STD", "125": "STD", "150": "STD", "200": "STD", "250": "STD", "300": "STD"}</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>{"15": "SCH40s", "20": "SCH40s", "25": "SCH40s", "32": "SCH40s", "40": "SCH40s", "50": "SCH10s", "65": "SCH10s", "80": "SCH10s", "100": "SCH10s", "150": "SCH10s", "200": "SCH10s", "250": "SCH10s", "300": "SCH10s"}</t>
+          <t>{"15": "SCH40s", "20": "SCH40s", "25": "SCH40s", "32": "SCH40s", "40": "SCH40s", "50": "SCH10s", "65": "SCH10s", "80": "SCH10s", "100": "SCH10s", "125": "SCH10s", "150": "SCH10s", "200": "SCH10s", "250": "SCH10s", "300": "SCH10s"}</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>{"15": "SCH40s", "20": "SCH40s", "25": "SCH40s", "32": "SCH40s", "40": "SCH40s", "50": "SCH10s", "65": "SCH10s", "80": "SCH10s", "100": "SCH10s", "150": "SCH10s", "200": "SCH10s", "250": "SCH10s", "300": "SCH10s", "350": "SCH10s", "400": "SCH10s", "450": "SCH10s", "500": "SCH10s", "600": "SCH10s"}</t>
+          <t>{"15": "SCH40s", "20": "SCH40s", "25": "SCH40s", "32": "SCH40s", "40": "SCH40s", "50": "SCH10s", "65": "SCH10s", "80": "SCH10s", "100": "SCH10s", "125": "SCH10s", "150": "SCH10s", "200": "SCH10s", "250": "SCH10s", "300": "SCH10s", "350": "SCH10s", "400": "SCH10s", "450": "SCH10s", "500": "SCH10s", "600": "SCH10s", "650": "SCH10s", "700": "SCH10s", "750": "SCH10s", "800": "SCH10", "850": "SCH10", "900": "SCH10"}</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">

</xml_diff>